<commit_message>
Stage 8 review fixes: A-018
</commit_message>
<xml_diff>
--- a/output/archive/VellacombeData/Clients/VP10/VD-26-068/Routes/Coupling/VP-C_screen_08Jul26_interim.xlsx
+++ b/output/archive/VellacombeData/Clients/VP10/VD-26-068/Routes/Coupling/VP-C_screen_08Jul26_interim.xlsx
@@ -19,9 +19,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -63,15 +61,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -167,17 +161,11 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Hassan Darwish</author>
-    <author>Ruth Calderwood</author>
   </authors>
   <commentList>
-    <comment ref="I3" authorId="0" shapeId="0">
+    <comment ref="C2" authorId="0" shapeId="0">
       <text>
-        <t>Conversions to go in once the HPLC runs are reviewed.</t>
-      </text>
-    </comment>
-    <comment ref="J5" authorId="1" shapeId="0">
-      <text>
-        <t>Repeat entry 4 with the T3P conditions at lower temperature before we drop this reagent.</t>
+        <t>Use the completed matrix in the route scout records; do not reconstruct individual conditions here.</t>
       </text>
     </comment>
   </commentList>
@@ -190,9 +178,9 @@
     <author>Clara Fenwick</author>
   </authors>
   <commentList>
-    <comment ref="E2" authorId="0" shapeId="0">
+    <comment ref="D2" authorId="0" shapeId="0">
       <text>
-        <t>Yield to be entered after drying overnight. Mass balance from the mother liquors goes in the note.</t>
+        <t>Transfer isolated mass and purity only after the trial record has been checked.</t>
       </text>
     </comment>
   </commentList>
@@ -592,7 +580,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>The coupling screen is logged in full on the next sheet. The isolation trials on the preferred solvent system are running, and the route will be chosen once their isolated material has been characterised. Entries marked [TBC] are not yet confirmed.</t>
+          <t>The coupling screen is complete. Consult the route scout records for the completed matrix and observations. Isolation trials continue on the preferred solvent system; final route selection remains open.</t>
         </is>
       </c>
     </row>
@@ -625,408 +613,77 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Entry</t>
+          <t>Record</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Acid partner</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Amine partner</t>
+          <t>Conditions</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Coupling reagent</t>
+          <t>Observations</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Solvent</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>Temp (°C)</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>Time (h)</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>Conversion (HPLC area %)</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
-        <is>
-          <t>Comment</t>
+          <t>Next step</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Coupling screen</t>
+        </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>VP-C acid</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Model amine</t>
+          <t>See completed route scout matrix</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>HATU</t>
+          <t>See route scout records</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>DIPEA</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>DMF</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="H2" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>[TBC]</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Clean by HPLC</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>VP-C acid</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Model amine</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>EDC / HOBt</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>NMM</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>DMF</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Slow; starting acid remains</t>
-        </is>
-      </c>
-    </row>
+          <t>Assess with isolation trials</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>VP-C acid</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Model amine</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>T3P</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Pyridine</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>EtOAc</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>[TBC]</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>VP-C acid</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Model amine</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>T3P</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Pyridine</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>EtOAc</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Epimerisation suspected; repeat at lower temperature</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>VP-C acid chloride</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Model amine</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Oxalyl chloride, then amine</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Et3N</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>DCM</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>VP-C acid</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Model amine</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>DIC / Oxyma</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>MeCN</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>[TBC]</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Solid precipitated during reaction</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>VP-C acid</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Model amine</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>HATU</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>DIPEA</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>MeCN</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>VP-C acid</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Model amine</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>EDC / HOBt</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>NMM</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>MeCN</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Not run to completion</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1041,22 +698,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Trial</t>
+          <t>Trial record</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
@@ -1066,25 +722,20 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Antisolvent</t>
+          <t>Scale (mg)</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Scale (mg)</t>
+          <t>Isolated mass (mg)</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Isolated yield (mg)</t>
+          <t>Purity (area %)</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Purity (area %)</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1093,117 +744,31 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>IT-1</t>
+          <t>See isolation trial records</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>EtOAc / heptane</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Heptane</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="E2" s="5" t="inlineStr"/>
-      <c r="F2" s="5" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Running</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>IT-2</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>EtOAc / heptane</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Heptane</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Queued</t>
-        </is>
-      </c>
-    </row>
+          <t>Preferred solvent system</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Continuing</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>IT-3</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>MeCN</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Water</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-    </row>
-    <row r="8">
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-    </row>
-    <row r="9">
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-    </row>
-    <row r="10">
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1274,7 +839,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Repeat coupling entry 4 at lower temperature</t>
+          <t>Review completed coupling screen alongside isolation trial records</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">

</xml_diff>